<commit_message>
Fix 21 Borrett Road / 波老道21号 district to Hong Kong Island - Mid-Levels West across all rule files
</commit_message>
<xml_diff>
--- a/项目商圈规则表.xlsx
+++ b/项目商圈规则表.xlsx
@@ -699,7 +699,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>港岛-半山区西部-21 Borrett Road</t>
+          <t>港岛-西半山-21 Borrett Road</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>港岛-半山区西部-应天</t>
+          <t>港岛-西半山-21 Borrett Road</t>
         </is>
       </c>
     </row>

</xml_diff>